<commit_message>
updated on 26th aug
</commit_message>
<xml_diff>
--- a/12603513.xlsx
+++ b/12603513.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/830e508683434252/Desktop/CAP776 Python- My Data My Code/12603513-MDMC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/830e508683434252/Desktop/CAP776 PYTHON MDMC/CAP776-PYTHON-MDMC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8412DEF-7BD0-46DE-921D-BEB2E487AF90}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53EDBD32-4E9C-4123-8576-AC1673F3E5DD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,18 @@
   </si>
   <si>
     <t>I have to give time on Python and SQL.</t>
+  </si>
+  <si>
+    <t>22-08-2026</t>
+  </si>
+  <si>
+    <t>CA is coming</t>
+  </si>
+  <si>
+    <t>23-08-2026</t>
+  </si>
+  <si>
+    <t>I have to work hard in C++</t>
   </si>
 </sst>
 </file>
@@ -516,6 +528,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1204,48 +1220,96 @@
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+      <c r="A10" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="14">
+        <v>420</v>
+      </c>
+      <c r="C10" s="14">
+        <v>45</v>
+      </c>
+      <c r="D10" s="14">
+        <v>240</v>
+      </c>
+      <c r="E10" s="14">
+        <v>120</v>
+      </c>
+      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>45</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
+        <v>570</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+      <c r="A11" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="14">
+        <v>360</v>
+      </c>
+      <c r="C11" s="14">
+        <v>60</v>
+      </c>
+      <c r="D11" s="14">
+        <v>180</v>
+      </c>
+      <c r="E11" s="14">
+        <v>60</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>30</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>690</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
+        <v>750</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>

</xml_diff>